<commit_message>
Sync rollup counts after the External File in Forms column fix
Multimedia 51/66 -> 52/66, total 262/355 (73.8%).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -6723,11 +6723,11 @@
       </c>
       <c r="J10" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (51/66)</t>
+          <t>Partial Coverage (52/66)</t>
         </is>
       </c>
       <c r="K10" s="0" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L10" s="0" t="n">
         <v>14</v>
@@ -7296,14 +7296,14 @@
         </is>
       </c>
       <c r="K27" s="0" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="L27" s="0" t="n">
         <v>93</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>73.7% automated (261/354 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro)</t>
+          <t>73.8% automated (262/355 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate Multimedia > Media 4 via already-proven attachment check
Its own note already said this was "technically approachable via
get_form_attachments(), already proven for Photo Verification/Image Resize
27-28, just never wired up" - true, just needed the CI invocation.
min-attachments=2 rather than 4, since the Media 2 submission it checks
has a best-effort video-recording step; confirmed live via a real recent
submission that audio/image/sign reliably attach, video does not.

Verified passing live locally before wiring into the existing Multimedia
Submit-History checks CI step. Rollup: Multimedia 52/66 -> 53/66, total
263/355 (74.1%).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -6723,14 +6723,14 @@
       </c>
       <c r="J10" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (52/66)</t>
+          <t>Partial Coverage (53/66)</t>
         </is>
       </c>
       <c r="K10" s="0" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L10" s="0" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" ht="45.75" customHeight="1" s="86">
@@ -7296,14 +7296,14 @@
         </is>
       </c>
       <c r="K27" s="0" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>73.8% automated (262/355 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro)</t>
+          <t>74.1% automated (263/355 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix a real undercount: merged cell in Updates (partial and failed)
Row 37 ("Update verification" - checks the app auto-updates to
V6/Version 22) is a real, distinct automated test case, but shares a
merged A-column cell with row 36 (both display "Update 17"). Every
prior count that relied on column A being non-blank to identify real
rows silently skipped it, undercounting this tab's automated total by
1 (26 -> 27, total 28 -> 29). Confirmed via a merged-cell scan across
every tracked tab that this is the only genuine instance (ExternalApp
Tests' own A4:A5 merge is a metadata label, not a test case row) -
the Master Plan sheet itself doesn't need any change, only this
rollup's counts did.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7123,11 +7123,11 @@
       <c r="I21" s="63" t="n"/>
       <c r="J21" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (26/28)</t>
+          <t>Partial Coverage (27/29)</t>
         </is>
       </c>
       <c r="K21" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L21" s="0" t="n">
         <v>2</v>
@@ -7296,14 +7296,14 @@
         </is>
       </c>
       <c r="K27" s="0" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L27" s="0" t="n">
         <v>82</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>77.2% automated (278/360 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro). CORRECTED (2026-09-17): the denominator was previously miscalculated as 355 without cross-checking against the sum of column L (Not Automatable Count, which sums to 82 excluding row 5) - 278+82=360 is the real total.</t>
+          <t>77.3% automated (279/361 test cases) - excludes Browserstack/Android Virtual Devices (35 test cases, already marked Not automatable/out of scope for Maestro)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Skip Custom Properties 15 on CommCare 2.65+, keep it for 2.64
2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), while
2.64 is still the current release. A flow tagged commcare_max_<major>_<minor>
now runs up to that version and is reported as skipped, with the reason, on a
newer APK (version from the release tag, else the APK manifest; unreadable ->
runs as before). No core flow carries the tag.

Workbooks: Custom Properties 15 noted as 2.64-and-earlier; Custom Properties 1
now passing in CI (72/209 automated, 16 left).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -8038,22 +8038,22 @@
       <c r="H16" s="98" t="n"/>
       <c r="I16" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Written, not yet passing: Custom Properties 1 (PIN offer / Set My PIN / PIN login - the first two live runs got through the PIN setup; the fixed PIN-login step hasn't been re-run) and Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed) - run by scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards (same set-then-restore approach as the core suite's hq_setup teardowns). Its HQ preparation worked live; the device runs were rejected by BrowserStack (HTTP 422, all parallel sessions busy) and still need a passing run. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
+          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. Written, not yet passing: Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed) - run by scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards. Its HQ preparation worked live; the device runs still need a passing run. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
         </is>
       </c>
       <c r="J16" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (11/20)</t>
+          <t>Partial Coverage (12/20)</t>
         </is>
       </c>
       <c r="K16" s="95" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L16" s="95" t="n">
         <v>4</v>
       </c>
       <c r="M16" s="95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N16" s="95" t="n">
         <v>20</v>
@@ -8217,17 +8217,17 @@
       </c>
       <c r="I20" s="101" t="inlineStr">
         <is>
-          <t>71 of 209 test cases automated so far; 17 more assessed automatable; 120 not automatable; the rest N/A.</t>
+          <t>72 of 209 test cases automated so far; 16 more assessed automatable; 120 not automatable; the rest N/A.</t>
         </is>
       </c>
       <c r="K20" s="100" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L20" s="100" t="n">
         <v>120</v>
       </c>
       <c r="M20" s="100" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N20" s="100" t="n">
         <v>209</v>

</xml_diff>

<commit_message>
Apply answers to the non-core open questions
Print from case detail is deprecated: remove the Print from Detail flows
and the pinned Basic Tests v1133 build they used; mark Print from Detail
1-4 N/A. Mapbox 2 confirmed N/A. Personal ID TC_01-03 (no test number for
the SMS OTP) and TC_37-42 (fingerprint) confirmed not automatable.
Graphing 20/22 confirmed as an HQ app configuration issue; the flow stays
blocked until the app is fixed. Workbooks updated: 69 of 85 feasible rows
automated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7384,7 +7384,8 @@
           <t>1. [Master] Mobile Plan (2026) - the 15 tabs not listed on the "CommCare Mobile" tab.
 2. Re-reviewed row by row on 2026-10-02 against the test steps, commcare-android source and the HQ apps themselves; several earlier notes were corrected (see each row). Automation for these tabs lives in flows_non_core/ and runs from its own workflow, .github/workflows/maestro-browserstack-non-core.yml - separate from the core flows/ suite.
 3. 'Tests Automated' counts only sheet rows covered by flows that passed a live BrowserStack run. 'Automatable - not yet automated' is the rest of what the review found automatable.
-4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.</t>
+4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.
+5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15 on 2.65+ still unanswered.</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7697,7 @@
       <c r="H9" s="98" t="n"/>
       <c r="I9" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/printing/ (all passed live): Form Printing 1-4 (fill Name/Age/Hometown, Get Data, Android's print UI opens), Print from Detail 1-2 (case detail shows Name/Status) and Print from Detail 3 (Print Case Detail opens the print UI). Finding: the current [Master] Basic Tests build ships the case-detail print template but no longer references it, so CommCare hides 'Print Case Detail' there (EntityDetailActivity, detail.isPrintEnabled()); Print from Detail 3 therefore runs on the pinned build v1133, which still has it - worth checking with the app owner whether dropping it was intended. Not automatable: Form Printing 5 and Print from Detail 4 (checking the PDF's contents).</t>
+          <t>Automated in flows_non_core/printing/ (all passed live): Form Printing 1-4 (fill Name/Age/Hometown, Get Data, Android's print UI opens). Print from Detail 1-4 are N/A: printing from the case detail is deprecated (confirmed with the team 2026-10-23), so the Print from Detail flows and the pinned v1133 build they used were removed from the suite. Not automatable: Form Printing 5 (checking the PDF's contents).</t>
         </is>
       </c>
       <c r="J9" s="95" t="inlineStr">
@@ -7705,10 +7706,10 @@
         </is>
       </c>
       <c r="K9" s="95" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L9" s="95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="95" t="n">
         <v>0</v>
@@ -7746,7 +7747,7 @@
       <c r="H10" s="98" t="n"/>
       <c r="I10" s="99" t="inlineStr">
         <is>
-          <t>Correction to the earlier note: graphs are NOT custom-drawn canvas - commcare-android renders them as c3/d3 SVG in a WebView (app/src/org/commcare/graph/view/GraphView.java), and Maestro can read their text (proven live). Automated in flows_non_core/graphing/ (passed live): Graphing 1-5, End Form 1, 19 (create case, add a point, view it, remove it - cleans up after itself), 6 (axis titles, tick labels zero/five/ten, BOTTOM, Secondary Y Values), 7-11 (each graph tab's titles/annotations: TOP, DateTime, JUNE, Fill Graph, Number One/Two, number2, Bar Horizontal Graph), 12 (double-tap opens the XY and Fill graphs full screen) and 18 (Remove a Point list with X/Y/Radius columns). Blocked on HQ, not tooling: Graphing 20/22 - the Add Details form submits, but 'User Info Reports' fails with CommCare's own 'Unable to find lookup table jr://fixture/commcare:reports' error (the app's mobile report fixture isn't restored to the test user); the flow is written and excluded from runs (blocked_app_config) until that's fixed. Not automatable: Graphing 13-17 and 21 (tap an individual data point - its screen position depends on device and data); colours, zoom/drag quality and rotation distortion in 6-12 stay visual.</t>
+          <t>Correction to the earlier note: graphs are NOT custom-drawn canvas - commcare-android renders them as c3/d3 SVG in a WebView (app/src/org/commcare/graph/view/GraphView.java), and Maestro can read their text (proven live). Automated in flows_non_core/graphing/ (passed live): Graphing 1-5, End Form 1, 19 (create case, add a point, view it, remove it - cleans up after itself), 6 (axis titles, tick labels zero/five/ten, BOTTOM, Secondary Y Values), 7-11 (each graph tab's titles/annotations: TOP, DateTime, JUNE, Fill Graph, Number One/Two, number2, Bar Horizontal Graph), 12 (double-tap opens the XY and Fill graphs full screen) and 18 (Remove a Point list with X/Y/Radius columns). Blocked on HQ, not tooling: Graphing 20/22 - the Add Details form submits, but 'User Info Reports' fails with CommCare's own 'Unable to find lookup table jr://fixture/commcare:reports' error (confirmed 2026-10-23 as an app configuration issue on HQ); the flow is written and excluded from runs (blocked_app_config) until the app is fixed. Not automatable: Graphing 13-17 and 21 (tap an individual data point - its screen position depends on device and data); colours, zoom/drag quality and rotation distortion in 6-12 stay visual.</t>
         </is>
       </c>
       <c r="J10" s="95" t="inlineStr">
@@ -7888,7 +7889,7 @@
       <c r="H13" s="98" t="n"/>
       <c r="I13" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/mapbox/ (all passed live): Mapbox 1 (GPS Normal capture), 4 (location permission denied via Maestro's launchApp permissions - CommCare re-asks and the capture completes once allowed) and 5 (new case in the Followup case list); the appearance='maps' question is captured too. Mapbox 2 is N/A on the current client: commcare-android removed Mapbox in 2.59.0 (commits 4607202fb / e6d3972c6), so 'maps' questions now open the Google-map picker - this tab of the Master Plan needs updating. Mapbox 3 (turn device GPS off system-wide) is not automatable.</t>
+          <t>Automated in flows_non_core/mapbox/ (all passed live): Mapbox 1 (GPS Normal capture), 4 (location permission denied via Maestro's launchApp permissions - CommCare re-asks and the capture completes once allowed) and 5 (new case in the Followup case list); the appearance='maps' question is captured too. Mapbox 2 is N/A (confirmed 2026-10-23): commcare-android removed Mapbox in 2.59.0 (commits 4607202fb / e6d3972c6), so 'maps' questions now open the Google-map picker. Mapbox 3 (turn device GPS off system-wide) is not automatable.</t>
         </is>
       </c>
       <c r="J13" s="95" t="inlineStr">
@@ -7900,7 +7901,7 @@
         <v>3</v>
       </c>
       <c r="L13" s="95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" s="95" t="n">
         <v>0</v>
@@ -8188,7 +8189,7 @@
       <c r="H19" s="98" t="n"/>
       <c r="I19" s="99" t="inlineStr">
         <is>
-          <t>Mostly the Connect/PersonalID product, not CommCare Mobile. Automated in flows_non_core/personal_id/ (passed live): TC_04 - 'Sign up for PersonalID' is offered in the login screen's menu (shown when nobody is signed in and the device passes PersonalID's compatibility check; it does on BrowserStack's Galaxy S26). TC_43-46 are HQ web checks (mobile workers page) - N/A for this mobile suite. The rest need a real SMS OTP or fingerprint enrollment and are counted Not automatable - but the Connect Mobile tab marks 'PersonalID Recovery' as already automated, which suggests the Connect team has a test-OTP path; if so, TC_01-03 and TC_37-42 become automatable. Worth asking them.</t>
+          <t>Mostly the Connect/PersonalID product, not CommCare Mobile. Automated in flows_non_core/personal_id/ (passed live): TC_04 - 'Sign up for PersonalID' is offered in the login screen's menu (shown when nobody is signed in and the device passes PersonalID's compatibility check; it does on BrowserStack's Galaxy S26). TC_43-46 are HQ web checks (mobile workers page) - N/A for this mobile suite. The rest are not automatable, confirmed with the team 2026-10-23: TC_01-03 need an SMS OTP and there is no test number that receives one; TC_37-42 need fingerprint enrollment.</t>
         </is>
       </c>
       <c r="J19" s="95" t="inlineStr">
@@ -8217,14 +8218,14 @@
       </c>
       <c r="I20" s="101" t="inlineStr">
         <is>
-          <t>72 of 209 test cases automated so far; 16 more assessed automatable; 120 not automatable; the rest N/A.</t>
+          <t>69 of 209 test cases automated so far; 16 more assessed automatable; 118 not automatable; the rest N/A.</t>
         </is>
       </c>
       <c r="K20" s="100" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L20" s="100" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M20" s="100" t="n">
         <v>16</v>

</xml_diff>

<commit_message>
Run targeted-updates and upgrade checks in non-core CI; add Database 6 and Database Change 13
- run_targeted_updates_check.py: pass 'Update to version N.*' instead of
  '... & log out' (BrowserStack's Maestro API 422s on '&' in env values),
  and retry HQ setup on a dropped connection. CP11-14 pass on 2.65.0.
- run_appium_non_core_upgrade_suite.py: match the 'Incomplete (1)' home
  tile. Database Change and Performance upgrades (2.45 -> 2.65.0) pass.
- Non-core workflow runs the targeted-updates check in group-a and the
  upgrade checks in group-b (or a matching single-tag dispatch).
- New flows: Database 6 (multimedia form saved, image + video) and
  Database Change 13 (Data Change Logs > Share > Gmail), both partial.
- Workbooks: 83 of 85 feasible non-core rows automated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7385,7 +7385,8 @@
 2. Re-reviewed row by row on 2026-10-02 against the test steps, commcare-android source and the HQ apps themselves; several earlier notes were corrected (see each row). Automation for these tabs lives in flows_non_core/ and runs from its own workflow, .github/workflows/maestro-browserstack-non-core.yml - separate from the core flows/ suite.
 3. 'Tests Automated' counts only sheet rows covered by flows that passed a live BrowserStack run. 'Automatable - not yet automated' is the rest of what the review found automatable.
 4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.
-5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15 on 2.65+ still unanswered.</t>
+5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15 on 2.65+ still unanswered.
+6. 2026-10-23: the targeted-updates and CommCare-upgrade runners passed live and now run in the non-core CI workflow; Database 6 and Database Change 13 were automated (partial).</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7486,7 @@
       </c>
       <c r="E5" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F5" s="98" t="inlineStr">
@@ -7497,22 +7498,22 @@
       <c r="H5" s="98" t="n"/>
       <c r="I5" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/database_change/ (passed live): Setup 2-3 and Database Change 10-12 - install the second most recent Basic Tests build (pinned v1139), update it to the current one, then App Manager &gt; Advanced &gt; Data Change Logs shows 'CommCare installed', 'App installed' and 'App updated' (messages from commcare-android DataChangeLog.kt). Written, awaiting a live run: scripts/run_appium_non_core_upgrade_suite.py --scenario database_change_upgrade covers Setup 1, Database 2, Final 1-2 and Database 7/9 - it installs CommCare 2.45 (resources/commcare_2.45_release.apk) with the 'Database Change!' app (its builds target CC 2.21, so 2.45 can install them; no Basic Tests build can), saves an incomplete form, upgrades CommCare to the release mid-session (BrowserStack Appium, same as the core Updates scenarios), then checks the form survived and Data Change Logs shows 'CommCare updated'. Not written yet: Database 6 (gallery parts) and Database Change 13 (Gmail share handoff). Not automatable: Setup 4 / Final 3 (airplane mode - network toggling on BrowserStack is a confirmed dead end) and therefore Database 1, 3, 4, 5 and Final 4 (without going offline the forms just submit); Database 8 needs Android 8 or lower (BrowserStack's minimum is 8.1).</t>
+          <t>Automated in flows_non_core/database_change/ (passed live): Setup 2-3 and Database Change 10-12 - install the second most recent Basic Tests build (pinned v1139), update it to the current one, then App Manager &gt; Advanced &gt; Data Change Logs shows 'CommCare installed', 'App installed' and 'App updated' (messages from commcare-android DataChangeLog.kt). Database 6 (partial): the Multimedia Only form with a gallery image and video, submitted, then reopened from Saved still lists both files (audio has no fixture; signature/acquire-only tiles need a companion app). Database Change 13 (partial): Data Change Logs &gt; Share &gt; Gmail opens Gmail - BrowserStack's devices have no Google account, so the draft/attachment and sending (steps 4-7) stay manual. Setup 1, Database 2, Final 1-2 and Database 7/9 (passed live 2026-10-23, 2.45 -&gt; 2.65.0): scripts/run_appium_non_core_upgrade_suite.py --scenario database_change_upgrade installs CommCare 2.45 (resources/commcare_2.45_release.apk) with the 'Database Change!' app, saves an incomplete form, upgrades CommCare to the release mid-session (BrowserStack Appium), then checks the form survived and Data Change Logs shows 'CommCare updated'; runs in the non-core workflow's group-b. Not automatable: Setup 4 / Final 3 (airplane mode - network toggling on BrowserStack is a confirmed dead end) and therefore Database 1, 3, 4, 5 and Final 4 (without going offline the forms just submit); Database 8 needs Android 8 or lower (BrowserStack's minimum is 8.1).</t>
         </is>
       </c>
       <c r="J5" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (5/21)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K5" s="95" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="L5" s="95" t="n">
         <v>8</v>
       </c>
       <c r="M5" s="95" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N5" s="95" t="n">
         <v>21</v>
@@ -8027,7 +8028,7 @@
       </c>
       <c r="E16" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F16" s="98" t="inlineStr">
@@ -8039,22 +8040,22 @@
       <c r="H16" s="98" t="n"/>
       <c r="I16" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. Written, not yet passing: Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed) - run by scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards. Its HQ preparation worked live; the device runs still need a passing run. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
+          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed, passed live 2026-10-23 on 2.65.0) run through scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards; it runs in the non-core workflow's group-a. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
         </is>
       </c>
       <c r="J16" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (12/20)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K16" s="95" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="L16" s="95" t="n">
         <v>4</v>
       </c>
       <c r="M16" s="95" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N16" s="95" t="n">
         <v>20</v>
@@ -8077,7 +8078,7 @@
       </c>
       <c r="E17" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F17" s="98" t="inlineStr">
@@ -8089,22 +8090,22 @@
       <c r="H17" s="98" t="n"/>
       <c r="I17" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/performance_tests/ (passed live): the two timing rows on Large App as the sheet's 'large' user - first run (2026-10-02, Galaxy S26 / Android 16): cold start to login screen 3.6 s, login to home screen ~114 s (includes the initial data restore). Times are reported on each CI run's summary page (scripts/extract_flow_timings.py); the budgets are loud-failure ceilings until real limits are agreed. Written, awaiting a live run: Perf 1-2 via scripts/run_appium_non_core_upgrade_suite.py --scenario performance_upgrade - CommCare 2.45 + Large App v194 (CC 2.41.1; 2.21 itself won't install on Android 10+), upgrade mid-session, then times both rows on the upgraded client. The 'large' user's password had drifted from the sheet's 123 and was reset to 123 on 2026-10-02.</t>
+          <t>Automated in flows_non_core/performance_tests/ (passed live): the two timing rows on Large App as the sheet's 'large' user - first run (2026-10-02, Galaxy S26 / Android 16): cold start to login screen 3.6 s, login to home screen ~114 s (includes the initial data restore). Times are reported on each CI run's summary page (scripts/extract_flow_timings.py); the budgets are loud-failure ceilings until real limits are agreed. Perf 1-2 (passed live 2026-10-23): scripts/run_appium_non_core_upgrade_suite.py --scenario performance_upgrade - CommCare 2.45 + Large App v194, upgraded mid-session to 2.65.0, then both timings on the upgraded client: cold start 2.0 s, login 57.8 s. Runs in the non-core workflow's group-b.</t>
         </is>
       </c>
       <c r="J17" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (2/4)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K17" s="95" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L17" s="95" t="n">
         <v>0</v>
       </c>
       <c r="M17" s="95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N17" s="95" t="n">
         <v>4</v>
@@ -8218,17 +8219,17 @@
       </c>
       <c r="I20" s="101" t="inlineStr">
         <is>
-          <t>69 of 209 test cases automated so far; 16 more assessed automatable; 118 not automatable; the rest N/A.</t>
+          <t>83 of 209 test cases automated so far; 2 more assessed automatable; 118 not automatable; the rest N/A.</t>
         </is>
       </c>
       <c r="K20" s="100" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="L20" s="100" t="n">
         <v>118</v>
       </c>
       <c r="M20" s="100" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="N20" s="100" t="n">
         <v>209</v>

</xml_diff>

<commit_message>
Graphing 20/22: run on a fixed copy of the Graphing app
The Graphing app's report graphs read the removed v1 report fixture
(instance('reports') = jr://fixture/commcare:reports) with v1 column
syntax, so they fail with 'Unable to find lookup table'. Run the flow on
'Graphing - Maestro Reports [DO NOT DELETE]' (GRAPHING_REPORTS), a copy
whose graphs use the v2 fixtures; the original app is unchanged. Legend
check follows the sheet (Age only). Workbooks: 85 of 85 feasible rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7386,7 +7386,8 @@
 3. 'Tests Automated' counts only sheet rows covered by flows that passed a live BrowserStack run. 'Automatable - not yet automated' is the rest of what the review found automatable.
 4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.
 5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15 on 2.65+ still unanswered.
-6. 2026-10-23: the targeted-updates and CommCare-upgrade runners passed live and now run in the non-core CI workflow; Database 6 and Database Change 13 were automated (partial).</t>
+6. 2026-10-23: the targeted-updates and CommCare-upgrade runners passed live and now run in the non-core CI workflow; Database 6 and Database Change 13 were automated (partial).
+7. 2026-10-27: Graphing 20/22 automated on a fixed copy of the Graphing app (see the Graphing row).</t>
         </is>
       </c>
     </row>
@@ -7736,7 +7737,7 @@
       </c>
       <c r="E10" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F10" s="98" t="inlineStr">
@@ -7748,22 +7749,22 @@
       <c r="H10" s="98" t="n"/>
       <c r="I10" s="99" t="inlineStr">
         <is>
-          <t>Correction to the earlier note: graphs are NOT custom-drawn canvas - commcare-android renders them as c3/d3 SVG in a WebView (app/src/org/commcare/graph/view/GraphView.java), and Maestro can read their text (proven live). Automated in flows_non_core/graphing/ (passed live): Graphing 1-5, End Form 1, 19 (create case, add a point, view it, remove it - cleans up after itself), 6 (axis titles, tick labels zero/five/ten, BOTTOM, Secondary Y Values), 7-11 (each graph tab's titles/annotations: TOP, DateTime, JUNE, Fill Graph, Number One/Two, number2, Bar Horizontal Graph), 12 (double-tap opens the XY and Fill graphs full screen) and 18 (Remove a Point list with X/Y/Radius columns). Blocked on HQ, not tooling: Graphing 20/22 - the Add Details form submits, but 'User Info Reports' fails with CommCare's own 'Unable to find lookup table jr://fixture/commcare:reports' error (confirmed 2026-10-23 as an app configuration issue on HQ); the flow is written and excluded from runs (blocked_app_config) until the app is fixed. Not automatable: Graphing 13-17 and 21 (tap an individual data point - its screen position depends on device and data); colours, zoom/drag quality and rotation distortion in 6-12 stay visual.</t>
+          <t>Correction to the earlier note: graphs are NOT custom-drawn canvas - commcare-android renders them as c3/d3 SVG in a WebView (app/src/org/commcare/graph/view/GraphView.java), and Maestro can read their text (proven live). Automated in flows_non_core/graphing/ (passed live): Graphing 1-5, End Form 1, 19 (create case, add a point, view it, remove it - cleans up after itself), 6 (axis titles, tick labels zero/five/ten, BOTTOM, Secondary Y Values), 7-11 (each graph tab's titles/annotations: TOP, DateTime, JUNE, Fill Graph, Number One/Two, number2, Bar Horizontal Graph), 12 (double-tap opens the XY and Fill graphs full screen) and 18 (Remove a Point list with X/Y/Radius columns). Graphing 20/22 (passed live 2026-10-27) run on 'Graphing - Maestro Reports [DO NOT DELETE]', a copy of the Graphing app made for automation: the original's two report graphs have custom series data paths on the removed v1 report fixture (instance('reports') = jr://fixture/commcare:reports, hence 'Unable to find lookup table') and v1 column syntax; the copy uses the v2 fixtures (instance('commcare-reports:&lt;report_slug&gt;')/rows/row, x/y column_0..2). The original app is unchanged - manual testers on it still hit the error until the same two edits are made there. Not automatable: Graphing 13-17 and 21 (tap an individual data point - its screen position depends on device and data); colours, zoom/drag quality and rotation distortion in 6-12 stay visual.</t>
         </is>
       </c>
       <c r="J10" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (15/23)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K10" s="95" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L10" s="95" t="n">
         <v>6</v>
       </c>
       <c r="M10" s="95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N10" s="95" t="n">
         <v>23</v>
@@ -8219,17 +8220,17 @@
       </c>
       <c r="I20" s="101" t="inlineStr">
         <is>
-          <t>83 of 209 test cases automated so far; 2 more assessed automatable; 118 not automatable; the rest N/A.</t>
+          <t>85 of 209 test cases automated so far; 0 more assessed automatable; 118 not automatable; the rest N/A.</t>
         </is>
       </c>
       <c r="K20" s="100" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L20" s="100" t="n">
         <v>118</v>
       </c>
       <c r="M20" s="100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N20" s="100" t="n">
         <v>209</v>

</xml_diff>

<commit_message>
Workbooks: Custom Properties 15 confirmed removed in 2.65 for good
Mobile dev confirmed root-menu-as-home-screen has no replacement; the
row and flow stay for 2.64 and earlier and can be retired with 2.64.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7385,7 +7385,7 @@
 2. Re-reviewed row by row on 2026-10-02 against the test steps, commcare-android source and the HQ apps themselves; several earlier notes were corrected (see each row). Automation for these tabs lives in flows_non_core/ and runs from its own workflow, .github/workflows/maestro-browserstack-non-core.yml - separate from the core flows/ suite.
 3. 'Tests Automated' counts only sheet rows covered by flows that passed a live BrowserStack run. 'Automatable - not yet automated' is the rest of what the review found automatable.
 4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.
-5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15 on 2.65+ still unanswered.
+5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15: removed in 2.65 for good (mobile dev, 2026-10-27) - kept for 2.64 and earlier only.
 6. 2026-10-23: the targeted-updates and CommCare-upgrade runners passed live and now run in the non-core CI workflow; Database 6 and Database Change 13 were automated (partial).
 7. 2026-10-27: Graphing 20/22 automated on a fixed copy of the Graphing app (see the Graphing row).</t>
         </is>
@@ -8041,7 +8041,7 @@
       <c r="H16" s="98" t="n"/>
       <c r="I16" s="99" t="inlineStr">
         <is>
-          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed, passed live 2026-10-23 on 2.65.0) run through scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards; it runs in the non-core workflow's group-a. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
+          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. The mobile dev confirmed 2026-10-27 that the feature is gone for good (no replacement), so the row and flow can be retired once 2.64 is no longer tested. Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed, passed live 2026-10-23 on 2.65.0) run through scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards; it runs in the non-core workflow's group-a. Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
         </is>
       </c>
       <c r="J16" s="95" t="inlineStr">

</xml_diff>

<commit_message>
Workbooks: refresh counts; add CommCare Mobile coverage table to Summary
Summary tab gets a test-case coverage block (core 279/361, non-core
85/209, total 364/570; 0 automatable left), read from the two tabs'
TOTAL rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -390,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -667,6 +667,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="86" min="1" max="1"/>
@@ -1130,12 +1131,124 @@
     </row>
     <row r="16" ht="14.25" customHeight="1" s="86"/>
     <row r="17" ht="14.25" customHeight="1" s="86"/>
-    <row r="18" ht="14.25" customHeight="1" s="86"/>
-    <row r="19" ht="14.25" customHeight="1" s="86"/>
-    <row r="20" ht="14.25" customHeight="1" s="86"/>
-    <row r="21" ht="14.25" customHeight="1" s="86"/>
-    <row r="22" ht="14.25" customHeight="1" s="86"/>
-    <row r="23" ht="14.25" customHeight="1" s="86"/>
+    <row r="18" ht="14.25" customHeight="1" s="86">
+      <c r="A18" s="102" t="inlineStr">
+        <is>
+          <t>CommCare Mobile - test-case automation coverage (Maestro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14.25" customHeight="1" s="86">
+      <c r="A19" s="94" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B19" s="94" t="inlineStr">
+        <is>
+          <t>Test Cases</t>
+        </is>
+      </c>
+      <c r="C19" s="94" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="D19" s="94" t="inlineStr">
+        <is>
+          <t>Not Automatable</t>
+        </is>
+      </c>
+      <c r="E19" s="94" t="inlineStr">
+        <is>
+          <t>Automatable - not yet automated</t>
+        </is>
+      </c>
+      <c r="F19" s="94" t="inlineStr">
+        <is>
+          <t>% of test cases automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14.25" customHeight="1" s="86">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>CommCare Mobile (core)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>361</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>279</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>82</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>77.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14.25" customHeight="1" s="86">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>CommCare Mobile - Non-Core</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>209</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>118</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>40.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14.25" customHeight="1" s="86">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B22" s="25" t="n">
+        <v>570</v>
+      </c>
+      <c r="C22" s="26" t="n">
+        <v>364</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>200</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="30" t="inlineStr">
+        <is>
+          <t>63.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14.25" customHeight="1" s="86">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Every automatable test case is automated (0 left). Updated 2026-10-27 from the TOTAL rows of the 'CommCare Mobile' and 'CommCare Mobile - Non-Core' tabs. Core excludes Browserstack/Android Virtual Devices (35 manual test cases). Non-Core 'Test Cases' also counts a few N/A rows (deprecated Print from Detail, Mapbox 2). Custom Properties 15 counts as automated but only applies to CommCare 2.64 and earlier - on 2.65+ it is not run and not counted in the run's totals (the feature was removed for good).</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="14.25" customHeight="1" s="86"/>
     <row r="25" ht="14.25" customHeight="1" s="86"/>
     <row r="26" ht="14.25" customHeight="1" s="86"/>
@@ -7298,6 +7411,7 @@
         <v>14</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="0" t="inlineStr">
         <is>
@@ -7391,6 +7505,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="69.75" customHeight="1" s="86">
       <c r="A4" s="94" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add non-core CommCare Mobile suite (flows_non_core/) with its own CI workflow (#5)
Non-core Master Mobile Plan tabs automated in flows_non_core/ with their own workflow (2 BrowserStack sessions, Saturdays 01:00 UTC), targeted-updates (manual dispatch only) and CommCare-upgrade runners, commcare_max_* version gate, release-APK lookup fix (also affects core), and workbook updates. 85/209 non-core test cases automated, 0 automatable left.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="38">
+  <fonts count="39">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -237,6 +237,11 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -385,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -658,6 +663,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="86" min="1" max="1"/>
@@ -1122,12 +1132,124 @@
     <row r="16" ht="14.25" customHeight="1" s="86"/>
     <row r="17" ht="14.25" customHeight="1" s="86"/>
     <row r="18" ht="14.25" customHeight="1" s="86"/>
-    <row r="19" ht="14.25" customHeight="1" s="86"/>
-    <row r="20" ht="14.25" customHeight="1" s="86"/>
-    <row r="21" ht="14.25" customHeight="1" s="86"/>
-    <row r="22" ht="14.25" customHeight="1" s="86"/>
-    <row r="23" ht="14.25" customHeight="1" s="86"/>
-    <row r="24" ht="14.25" customHeight="1" s="86"/>
+    <row r="19" ht="14.25" customHeight="1" s="86">
+      <c r="A19" s="102" t="inlineStr">
+        <is>
+          <t>CommCare Mobile - test-case automation coverage (Maestro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14.25" customHeight="1" s="86">
+      <c r="A20" s="94" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B20" s="94" t="inlineStr">
+        <is>
+          <t>Test Cases</t>
+        </is>
+      </c>
+      <c r="C20" s="94" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="D20" s="94" t="inlineStr">
+        <is>
+          <t>Not Automatable</t>
+        </is>
+      </c>
+      <c r="E20" s="94" t="inlineStr">
+        <is>
+          <t>Automatable - not yet automated</t>
+        </is>
+      </c>
+      <c r="F20" s="94" t="inlineStr">
+        <is>
+          <t>% of test cases automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14.25" customHeight="1" s="86">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>CommCare Mobile (core)</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>361</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>279</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>82</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>77.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14.25" customHeight="1" s="86">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>CommCare Mobile - Non-Core</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>209</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>118</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>40.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14.25" customHeight="1" s="86">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="n">
+        <v>570</v>
+      </c>
+      <c r="C23" s="26" t="n">
+        <v>364</v>
+      </c>
+      <c r="D23" s="28" t="n">
+        <v>200</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="30" t="inlineStr">
+        <is>
+          <t>63.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14.25" customHeight="1" s="86">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Every automatable test case is automated (0 left). Updated 2026-10-27 from the TOTAL rows of the 'CommCare Mobile' and 'CommCare Mobile - Non-Core' tabs. Core excludes Browserstack/Android Virtual Devices (35 manual test cases). Non-Core 'Test Cases' also counts a few N/A rows (deprecated Print from Detail, Mapbox 2). Custom Properties 15 counts as automated but only applies to CommCare 2.64 and earlier - on 2.65+ it is not run and not counted in the run's totals (the feature was removed for good).</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="14.25" customHeight="1" s="86"/>
     <row r="26" ht="14.25" customHeight="1" s="86"/>
     <row r="27" ht="14.25" customHeight="1" s="86"/>
@@ -7289,6 +7411,7 @@
         <v>14</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="0" t="inlineStr">
         <is>
@@ -7343,7 +7466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.71" customWidth="1" style="86" min="1" max="1"/>
@@ -7356,6 +7479,10 @@
     <col width="24" customWidth="1" style="86" min="8" max="8"/>
     <col width="37.29" customWidth="1" style="86" min="9" max="9"/>
     <col width="26" customWidth="1" style="86" min="10" max="10"/>
+    <col width="14" customWidth="1" style="86" min="11" max="11"/>
+    <col width="14" customWidth="1" style="86" min="12" max="12"/>
+    <col width="14" customWidth="1" style="86" min="13" max="13"/>
+    <col width="14" customWidth="1" style="86" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7368,12 +7495,17 @@
     <row r="2" ht="130" customHeight="1" s="86">
       <c r="A2" s="93" t="inlineStr">
         <is>
-          <t>1. [Master] Mobile Plan (2026) - 15 sheets not yet listed in the "CommCare Mobile" tab above
-2. Existing Unit Tests coverage
-These 15 tabs predate/sit outside the Maestro automation program - confirmed 2026-09-01 that none of them even carry a "Maestro Automatability" column in the Master Plan (unlike every tab in the "CommCare Mobile" sheet above). Reviewed here for the first time against this program's actual proven capabilities (HQClient's mark_build_status/create_new_build/set_custom_properties/get_custom_properties/list_releases/get_app_install_code/find_recent_submission+get_form_metadata/edit_module_attr/check_for_phone_triggered_build; Appium's push_file/current_package/mid-session same-cert app install; confirmed dead ends: camera-image-injection, airplane-mode/network toggling on BrowserStack's real-device cloud, arbitrary third-party Play Store app installs with no internal APK source, device-clock manipulation, biometric hardware enrollment, real SMS OTP delivery, terminateApp/backgroundApp/pressKeyCode/adb_shell).</t>
-        </is>
-      </c>
-    </row>
+          <t>1. [Master] Mobile Plan (2026) - the 15 tabs not listed on the "CommCare Mobile" tab.
+2. Re-reviewed row by row on 2026-10-02 against the test steps, commcare-android source and the HQ apps themselves; several earlier notes were corrected (see each row). Automation for these tabs lives in flows_non_core/ and runs from its own workflow, .github/workflows/maestro-browserstack-non-core.yml - separate from the core flows/ suite.
+3. 'Tests Automated' counts only sheet rows covered by flows that passed a live BrowserStack run. 'Automatable - not yet automated' is the rest of what the review found automatable.
+4. Row-level status is also in each of these 15 Master Plan tabs, columns I/J/K (Maestro Automatability / Automated? / Flow File) - the same columns the core tabs use. Second re-scan 2026-10-02 added Graphing 6-12/18, Print from Detail 3, Database Change 10-12, Custom Properties 1, Third Party Scanner 2/6 and Personal ID TC_04.
+5. Open questions answered 2026-10-23: Print from Detail is deprecated (rows N/A, flows removed); Mapbox 2 N/A; Personal ID TC_01-03 (no test OTP number) and TC_37-42 (fingerprint) not automatable; Graphing 20/22 are an HQ app configuration issue (flow kept, blocked until the app is fixed); Custom Properties 15: removed in 2.65 for good (mobile dev, 2026-10-27) - kept for 2.64 and earlier only.
+6. 2026-10-23: the targeted-updates and CommCare-upgrade runners passed live and now run in the non-core CI workflow (targeted updates on manual dispatch only, from 2026-10-28); Database 6 and Database Change 13 were automated (partial).
+7. 2026-10-27: Graphing 20/22 automated on a fixed copy of the Graphing app (see the Graphing row).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="69.75" customHeight="1" s="86">
       <c r="A4" s="94" t="inlineStr">
         <is>
@@ -7424,6 +7556,32 @@
         <is>
           <t>Notes / Dependencies
 (CommCare dev needed? blocker? volatile?)</t>
+        </is>
+      </c>
+      <c r="J4" s="94" t="inlineStr">
+        <is>
+          <t>Maestro Automated
+(Yes / Partial Coverage / No / N/A)</t>
+        </is>
+      </c>
+      <c r="K4" s="94" t="inlineStr">
+        <is>
+          <t>Tests Automated (Count)</t>
+        </is>
+      </c>
+      <c r="L4" s="94" t="inlineStr">
+        <is>
+          <t>Not Automatable (Count)</t>
+        </is>
+      </c>
+      <c r="M4" s="94" t="inlineStr">
+        <is>
+          <t>Automatable - not yet automated (Count)</t>
+        </is>
+      </c>
+      <c r="N4" s="94" t="inlineStr">
+        <is>
+          <t>Test Cases (Count)</t>
         </is>
       </c>
     </row>
@@ -7444,16 +7602,37 @@
       </c>
       <c r="E5" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F5" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/database_change/</t>
+        </is>
+      </c>
       <c r="G5" s="98" t="n"/>
       <c r="H5" s="98" t="n"/>
       <c r="I5" s="99" t="inlineStr">
         <is>
-          <t>Tests local DB survives a CommCare/app-build upgrade (incl. large version jumps), with outstanding saved/incomplete/case/multimedia data preserved and submittable after update. Setup 2-4 and Database 1-6 (offline form creation, standard Maestro) and Final 3-4 (disable airplane mode, sync, verify via HQClient.find_recent_submission) are automatable now. The version-jump rows don't need real Play Store access either - install_mid_session can push the target GitHub-release APK directly (same signing cert). Database Change Logs (10-12) are plain text assertions. Row 13 (Share via Gmail) - handoff confirmable via driver.current_package, actual email delivery/contents out of scope. No instrumentation-test overlap (SyncRecoveryTest.kt covers mid-sync recovery within one app version, not cross-version DB migration).</t>
-        </is>
+          <t>Automated in flows_non_core/database_change/ (passed live): Setup 2-3 and Database Change 10-12 - install the second most recent Basic Tests build (pinned v1139), update it to the current one, then App Manager &gt; Advanced &gt; Data Change Logs shows 'CommCare installed', 'App installed' and 'App updated' (messages from commcare-android DataChangeLog.kt). Database 6 (partial): the Multimedia Only form with a gallery image and video, submitted, then reopened from Saved still lists both files (audio has no fixture; signature/acquire-only tiles need a companion app). Database Change 13 (partial): Data Change Logs &gt; Share &gt; Gmail opens Gmail - BrowserStack's devices have no Google account, so the draft/attachment and sending (steps 4-7) stay manual. Setup 1, Database 2, Final 1-2 and Database 7/9 (passed live 2026-10-23, 2.45 -&gt; 2.65.0): scripts/run_appium_non_core_upgrade_suite.py --scenario database_change_upgrade installs CommCare 2.45 (resources/commcare_2.45_release.apk) with the 'Database Change!' app, saves an incomplete form, upgrades CommCare to the release mid-session (BrowserStack Appium), then checks the form survived and Data Change Logs shows 'CommCare updated'; runs in the non-core workflow's group-b. Not automatable: Setup 4 / Final 3 (airplane mode - network toggling on BrowserStack is a confirmed dead end) and therefore Database 1, 3, 4, 5 and Final 4 (without going offline the forms just submit); Database 8 needs Android 8 or lower (BrowserStack's minimum is 8.1).</t>
+        </is>
+      </c>
+      <c r="J5" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" s="95" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="95" t="n">
+        <v>8</v>
+      </c>
+      <c r="M5" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="95" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="6" ht="90" customHeight="1" s="86">
@@ -7473,16 +7652,37 @@
       </c>
       <c r="E6" s="98" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/sd_card_dump/</t>
+        </is>
+      </c>
       <c r="G6" s="98" t="n"/>
       <c r="H6" s="98" t="n"/>
       <c r="I6" s="99" t="inlineStr">
         <is>
-          <t>Not automatable, out of scope: requires TWO physical Android phones, each with a real SD card slot, plus physically removing/inserting an SD card between them to transfer forms. BrowserStack App Automate is single-real-device-per-session with no way to move physical removable media. No instrumentation overlap.</t>
-        </is>
+          <t>Needs two phones with SD card slots and physically moving the card - out of scope. Exception, automated in flows_non_core/sd_card_dump/: SD Card 1 (Advanced &gt; Manage SD shows the 'Form Dump' warning, then the Dump/Submit screen) - single-device, passed live.</t>
+        </is>
+      </c>
+      <c r="J6" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" s="95" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="95" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="95" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1" s="86">
@@ -7502,16 +7702,37 @@
       </c>
       <c r="E7" s="98" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/wifi_direct/</t>
+        </is>
+      </c>
       <c r="G7" s="98" t="n"/>
       <c r="H7" s="98" t="n"/>
       <c r="I7" s="99" t="inlineStr">
         <is>
-          <t>Not automatable, out of scope: requires two physical devices to peer-connect via Wi-Fi Direct and transfer forms device-to-device - inherently a two-real-device session a single-device cloud service cannot provide. No instrumentation overlap.</t>
-        </is>
+          <t>Needs two devices peer-connected over Wi-Fi Direct - out of scope. Exception, automated in flows_non_core/wifi_direct/: WiFi 1 (Advanced &gt; Wi-Fi Direct opens the Send/Receive/Submit dialog and switches mode) - single-device, passed live.</t>
+        </is>
+      </c>
+      <c r="J7" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" s="95" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="95" t="n">
+        <v>7</v>
+      </c>
+      <c r="M7" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="95" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" s="86">
@@ -7531,16 +7752,37 @@
       </c>
       <c r="E8" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F8" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F8" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/developer_options/</t>
+        </is>
+      </c>
       <c r="G8" s="98" t="n"/>
       <c r="H8" s="98" t="n"/>
       <c r="I8" s="99" t="inlineStr">
         <is>
-          <t>Fully automatable in principle (single device, standard taps/asserts, no HQ/multi-device dependency) - and largely ALREADY covered, just not in this repo: commcare-android's DeveloperOptionsTests.kt (instrumentation) already exercises enabling Developer Mode and all 4 settings items (DO1), the Show Update Options toggle (DO2), and Image Above/Below Question Text with real Espresso isAbove/isBelow layout assertions (DO3/DO4) almost verbatim against this same sheet.</t>
-        </is>
+          <t>Automated in flows_non_core/developer_options/: do_01 (Setup 1-2 + DO1, all four option items), do_03 / do_04 (image above / below the question label, checked with Maestro's above/below position matchers - the same isAbove/isBelow checks commcare-android's DeveloperOptionsTests.kt makes). DO2 only says 'run the Update tab' - covered there, counted N/A here.</t>
+        </is>
+      </c>
+      <c r="J8" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" s="95" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="95" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1" s="86">
@@ -7560,16 +7802,37 @@
       </c>
       <c r="E9" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F9" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F9" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/printing/</t>
+        </is>
+      </c>
       <c r="G9" s="98" t="n"/>
       <c r="H9" s="98" t="n"/>
       <c r="I9" s="99" t="inlineStr">
         <is>
-          <t>Install/navigate/select-case steps are ordinary Maestro navigation. PDF generation (native Android print spooler UI) and verifying entered values appear correctly in the downloaded PDF are out of scope for a real tooling reason (not hardware): no file-content/PDF-rendering verification path exists in this repo's toolset, and the print spooler UI is largely outside Espresso/Maestro's reach. Instrumentation overlap is tangential only (AppPreferenceSettingsTest.kt's Set Print Template test picks a template FILE, not this sheet's PDF-output verification).</t>
-        </is>
+          <t>Automated in flows_non_core/printing/ (all passed live): Form Printing 1-4 (fill Name/Age/Hometown, Get Data, Android's print UI opens). Print from Detail 1-4 are N/A: printing from the case detail is deprecated (confirmed with the team 2026-10-23), so the Print from Detail flows and the pinned v1133 build they used were removed from the suite. Not automatable: Form Printing 5 (checking the PDF's contents).</t>
+        </is>
+      </c>
+      <c r="J9" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" s="95" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="95" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1" s="86">
@@ -7589,16 +7852,37 @@
       </c>
       <c r="E10" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F10" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/graphing/</t>
+        </is>
+      </c>
       <c r="G10" s="98" t="n"/>
       <c r="H10" s="98" t="n"/>
       <c r="I10" s="99" t="inlineStr">
         <is>
-          <t>Install/login/create-case/add-points navigation (Graphing 1-5) is plain Maestro. The real assertions (exact axis tick values, bar/bubble colors, zoom/pan/rotation not distorting) are out of scope for a genuine tooling reason: pixel/visual-rendering checks on a custom-drawn canvas, not accessibility-tree text Maestro can assert. No instrumentation overlap (TilesTest.kt tests an unrelated case-list UI).</t>
-        </is>
+          <t>Correction to the earlier note: graphs are NOT custom-drawn canvas - commcare-android renders them as c3/d3 SVG in a WebView (app/src/org/commcare/graph/view/GraphView.java), and Maestro can read their text (proven live). Automated in flows_non_core/graphing/ (passed live): Graphing 1-5, End Form 1, 19 (create case, add a point, view it, remove it - cleans up after itself), 6 (axis titles, tick labels zero/five/ten, BOTTOM, Secondary Y Values), 7-11 (each graph tab's titles/annotations: TOP, DateTime, JUNE, Fill Graph, Number One/Two, number2, Bar Horizontal Graph), 12 (double-tap opens the XY and Fill graphs full screen) and 18 (Remove a Point list with X/Y/Radius columns). Graphing 20/22 (passed live 2026-10-27) run on 'Graphing - Maestro Reports [DO NOT DELETE]', a copy of the Graphing app made for automation: the original's two report graphs have custom series data paths on the removed v1 report fixture (instance('reports') = jr://fixture/commcare:reports, hence 'Unable to find lookup table') and v1 column syntax; the copy uses the v2 fixtures (instance('commcare-reports:&lt;report_slug&gt;')/rows/row, x/y column_0..2). The original app is unchanged - manual testers on it still hit the error until the same two edits are made there. Not automatable: Graphing 13-17 and 21 (tap an individual data point - its screen position depends on device and data); colours, zoom/drag quality and rotation distortion in 6-12 stay visual.</t>
+        </is>
+      </c>
+      <c r="J10" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="95" t="n">
+        <v>17</v>
+      </c>
+      <c r="L10" s="95" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="95" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="11" ht="90" customHeight="1" s="86">
@@ -7626,8 +7910,25 @@
       <c r="H11" s="98" t="n"/>
       <c r="I11" s="99" t="inlineStr">
         <is>
-          <t>Not automatable, out of scope - the sheet's own header states this can only be run on a specific NFC-capable tablet physically located at a specific Dimagi office, tapped against a physical NFC bracelet. No BrowserStack cloud device offers this. No instrumentation overlap.</t>
-        </is>
+          <t>Not automatable (16 test rows - the earlier count of 14 was wrong): only runs on the NFC-capable tablet in the Dimagi office, tapped against a physical NFC bracelet. No cloud device offers this.</t>
+        </is>
+      </c>
+      <c r="J11" s="95" t="inlineStr">
+        <is>
+          <t>N/A - not automatable</t>
+        </is>
+      </c>
+      <c r="K11" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="95" t="n">
+        <v>16</v>
+      </c>
+      <c r="M11" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="95" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1" s="86">
@@ -7655,8 +7956,25 @@
       <c r="H12" s="98" t="n"/>
       <c r="I12" s="99" t="inlineStr">
         <is>
-          <t>Not automatable, out of scope: relies on airplane-mode/network toggling (confirmed unreliable on BrowserStack's real-device cloud this session) AND simulating a specific low-battery device state, neither of which this stack can do. No instrumentation overlap.</t>
-        </is>
+          <t>Not automatable: needs airplane-mode/network toggling (a confirmed BrowserStack dead end), a low-battery device state, and an hour-plus unattended wait.</t>
+        </is>
+      </c>
+      <c r="J12" s="95" t="inlineStr">
+        <is>
+          <t>N/A - not automatable</t>
+        </is>
+      </c>
+      <c r="K12" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="95" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="95" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="90" customHeight="1" s="86">
@@ -7676,16 +7994,37 @@
       </c>
       <c r="E13" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F13" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/mapbox/</t>
+        </is>
+      </c>
       <c r="G13" s="98" t="n"/>
       <c r="H13" s="98" t="n"/>
       <c r="I13" s="99" t="inlineStr">
         <is>
-          <t>Mapbox 1, 2, 5 (map-style rendering, case-list geopoint display) are standard Maestro taps/asserts on real UI elements. Mapbox 3-4 (disable device GPS / deny location permission via the real Android Settings app) are plausibly reachable via ordinary taps but unproven in this repo - flag as lower-confidence, not assumed reliable, until tried live. No instrumentation overlap (no GPS/location logic in the 35 files).</t>
-        </is>
+          <t>Automated in flows_non_core/mapbox/ (all passed live): Mapbox 1 (GPS Normal capture), 4 (location permission denied via Maestro's launchApp permissions - CommCare re-asks and the capture completes once allowed) and 5 (new case in the Followup case list); the appearance='maps' question is captured too. Mapbox 2 is N/A (confirmed 2026-10-23): commcare-android removed Mapbox in 2.59.0 (commits 4607202fb / e6d3972c6), so 'maps' questions now open the Google-map picker. Mapbox 3 (turn device GPS off system-wide) is not automatable.</t>
+        </is>
+      </c>
+      <c r="J13" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" s="95" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="95" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="95" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="14" ht="90" customHeight="1" s="86">
@@ -7705,16 +8044,37 @@
       </c>
       <c r="E14" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F14" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/text_to_speech/</t>
+        </is>
+      </c>
       <c r="G14" s="98" t="n"/>
       <c r="H14" s="98" t="n"/>
       <c r="I14" s="99" t="inlineStr">
         <is>
-          <t>TTS 1-4 (enable setting, audio-button presence, language-switch persistence) are standard taps/asserts. TTS 5-6 (delete/add on-device Google TTS language packs via native OEM TTS engine settings) vary across BrowserStack's device pool - not reliably automatable, skip. LanguagesTest.kt covers app-language-change persistence generically but has no TTS/audio-button assertions - tangential, not real coverage.</t>
-        </is>
+          <t>Automated (partial) in flows_non_core/text_to_speech/ (all passed live): TTS 1-2 (enable the setting; audio button shows and can be tapped), TTS 3 (form language switched to Hindi - label changes, button stays), TTS 4 (app language switched to Hindi, same check). We can't check that speech actually plays or is in Hindi. TTS 5-6 need on-device language packs downloaded/deleted through the OEM TTS engine settings - not reliable across BrowserStack devices.</t>
+        </is>
+      </c>
+      <c r="J14" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="95" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="95" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="90" customHeight="1" s="86">
@@ -7734,16 +8094,37 @@
       </c>
       <c r="E15" s="98" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/third_party_scanner/</t>
+        </is>
+      </c>
       <c r="G15" s="98" t="n"/>
       <c r="H15" s="98" t="n"/>
       <c r="I15" s="99" t="inlineStr">
         <is>
-          <t>Not automatable, out of scope: the entire premise (row 1: "Open Play Store, download QR Droid") requires installing an arbitrary third-party Play Store app with no internal APK source - a confirmed hard limit of this pipeline (same class of gap as Other-Error Tests' Callout Setup/Arbitrary Intent rows). No instrumentation overlap.</t>
-        </is>
+          <t>Rows 1, 3-5 and 7 need a third-party scanner app installed from the Play Store (no internal APK) - not automatable. Automated in flows_non_core/third_party_scanner/ (passed live): row 2 (toggle 'Use intent callout for scanner') and row 6 (with it disabled, the barcode question's Get Barcode opens CommCare's built-in scanner). With no third-party app installed CommCare falls back to the built-in ZXing scanner either way (WidgetUtils.createScanIntent), so the flow checks the setting and that the scanner launches, not which one.</t>
+        </is>
+      </c>
+      <c r="J15" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" s="95" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="95" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="95" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="16" ht="90" customHeight="1" s="86">
@@ -7763,16 +8144,37 @@
       </c>
       <c r="E16" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F16" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F16" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/advanced_settings/</t>
+        </is>
+      </c>
       <c r="G16" s="98" t="n"/>
       <c r="H16" s="98" t="n"/>
       <c r="I16" s="99" t="inlineStr">
         <is>
-          <t>Strongly automatable: most Custom Properties rows (1,2,4-9,11-16) map directly onto the proven HQClient.set_custom_properties/get_custom_properties mechanism plus a standard on-device assertion of the resulting UI. Settings 1/3/4 are plain UI assertions. Custom Properties 3 (device-clock change) and Settings 2 (device-date change) are blocked - real device-clock manipulation is a confirmed hard limit. Real instrumentation overlap: DeveloperOptionsTests.kt exercises the exact cc-superuser-enabled -&gt; Developer Options flow (Custom Properties 4); MediaEncryptionTest.kt directly toggles HiddenPreferences.ENCRYPT_CAPTURED_MEDIA, matching cc-encrypt-captured-media (Custom Properties 16).</t>
-        </is>
+          <t>Automated in flows_non_core/advanced_settings/ against the 'Advanced Settings' app (its custom properties are already set on HQ - nothing is changed there), all passed live: Custom Properties 1 (PIN offer, don't-ask-again, Set My PIN, PIN login), 2, 4, 5, 6, 7, 8, 9, 10, 15 and Settings 1, 4. Custom Properties 15 applies to CommCare 2.64 and earlier only: 2.65 deleted root-menu-as-home-screen (commcare-android 568e15b6d), so the flow is tagged commcare_max_2_64 and reported as skipped, with the reason, on 2.65+ APKs. The mobile dev confirmed 2026-10-27 that the feature is gone for good (no replacement), so the row and flow can be retired once 2.64 is no longer tested. Custom Properties 11-14 (cc-update-target release/build/save and pre-update-sync-needed, passed live 2026-10-23 on 2.65.0) run through scripts/run_targeted_updates_check.py, which sets the Targeted Updates App's custom properties on HQ, cuts the builds each row needs, runs the flow and restores the app's original settings + a clean released build afterwards; in CI it runs only on a manual dispatch with 'run_targeted_updates' ticked (not the Saturday schedule - each run cuts ~9 builds on HQ that can't be deleted). Not automatable: Custom Properties 3, Settings 2, Settings 3 (they change the device clock/date) and Custom Properties 16 (its check is that captured media files on the device end in .aes - listing app files needs adb_shell, which BrowserStack disables).</t>
+        </is>
+      </c>
+      <c r="J16" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K16" s="95" t="n">
+        <v>16</v>
+      </c>
+      <c r="L16" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="M16" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="95" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="17" ht="90" customHeight="1" s="86">
@@ -7792,16 +8194,37 @@
       </c>
       <c r="E17" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F17" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F17" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/performance_tests/</t>
+        </is>
+      </c>
       <c r="G17" s="98" t="n"/>
       <c r="H17" s="98" t="n"/>
       <c r="I17" s="99" t="inlineStr">
         <is>
-          <t>Install-old-APK-then-update matches the proven mid-session app-install pattern (AppiumBrowserStackClient.install_mid_session, same-signing-cert APKs, already used for update scenarios). "Time taken" rows are measurable via code-level timestamps around driver actions instead of a human stopwatch - no fundamental hardware blocker. No instrumentation overlap (no timing/perf measurement in the 35 files).</t>
-        </is>
+          <t>Automated in flows_non_core/performance_tests/ (passed live): the two timing rows on Large App as the sheet's 'large' user - first run (2026-10-02, Galaxy S26 / Android 16): cold start to login screen 3.6 s, login to home screen ~114 s (includes the initial data restore). Times are reported on each CI run's summary page (scripts/extract_flow_timings.py); the budgets are loud-failure ceilings until real limits are agreed. Perf 1-2 (passed live 2026-10-23): scripts/run_appium_non_core_upgrade_suite.py --scenario performance_upgrade - CommCare 2.45 + Large App v194, upgraded mid-session to 2.65.0, then both timings on the upgraded client: cold start 2.0 s, login 57.8 s. Runs in the non-core workflow's group-b.</t>
+        </is>
+      </c>
+      <c r="J17" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K17" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="95" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="18" ht="90" customHeight="1" s="86">
@@ -7821,16 +8244,37 @@
       </c>
       <c r="E18" s="98" t="inlineStr">
         <is>
-          <t>Partial Coverage</t>
-        </is>
-      </c>
-      <c r="F18" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F18" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/case_list_optimization/</t>
+        </is>
+      </c>
       <c r="G18" s="98" t="n"/>
       <c r="H18" s="98" t="n"/>
       <c r="I18" s="99" t="inlineStr">
         <is>
-          <t>Setup/Cache-and-index/Load-time rows are automatable via timestamped navigation (same technique as Performance Tests above). Load-time-6 (clear app data) and -7 (force-stop) are blocked: terminateApp/pressKeyCode are confirmed unsupported via Appium on BrowserStack, and its managed Appium server has adb_shell disabled - no way to force-stop or clear data. The Exploratory-testing row is inherently manual. Instrumentation overlap is weak (CaseListSortTest.kt/CaseListSearchTest.kt test sort/search correctness on a different app, not this sheet's cache/lazy-load performance settings).</t>
-        </is>
+          <t>Automated in flows_non_core/case_list_optimization/ (all passed live): Setup 1-2, Cache and index-1/2 (lists load; sort-order check not done yet) and Load time-1..8, each timed in code with a loud-failure ceiling (60 s) until real limits are agreed. Times appear on each CI run's summary page (scripts/extract_flow_timings.py) - first live run: Load time-1 3.1 s, Cache and index-1 3.0 s, -2 2.9 s. Correction to the earlier note: Load time-6 (clear app data) and -7 (force stop) are NOT blocked - those limits were Appium's; Maestro's own clearState and stopApp both work on BrowserStack (passed live). Exploratory testing stays manual. Runs as the sheet's '123' user (CC_CASELIST_USERNAME/PASSWORD).</t>
+        </is>
+      </c>
+      <c r="J18" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" s="95" t="n">
+        <v>13</v>
+      </c>
+      <c r="L18" s="95" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="95" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="19" ht="90" customHeight="1" s="86">
@@ -7850,16 +8294,61 @@
       </c>
       <c r="E19" s="98" t="inlineStr">
         <is>
-          <t>No - wrong product for most rows</t>
-        </is>
-      </c>
-      <c r="F19" s="98" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F19" s="98" t="inlineStr">
+        <is>
+          <t>flows_non_core/personal_id/</t>
+        </is>
+      </c>
       <c r="G19" s="98" t="n"/>
       <c r="H19" s="98" t="n"/>
       <c r="I19" s="99" t="inlineStr">
         <is>
-          <t>Mostly does not belong in a CommCare Mobile inventory: TC_05-36 are Dimagi Connect/PersonalID's own onboarding UI (phone OTP verification, Android biometric enrollment, backup codes, selfie capture) - a different product surface. Only TC_01-04 (existing-user sign-in/update continuity) and TC_37-47 (MW-to-PersonalID link/unlink popups inside CommCare, HQ mobile-workers-page column) genuinely touch CommCare Mobile, and even those are doubly blocked where they depend on real SMS OTP delivery or biometric hardware enrollment - two more confirmed hard limits. No instrumentation overlap.</t>
-        </is>
+          <t>Mostly the Connect/PersonalID product, not CommCare Mobile. Automated in flows_non_core/personal_id/ (passed live): TC_04 - 'Sign up for PersonalID' is offered in the login screen's menu (shown when nobody is signed in and the device passes PersonalID's compatibility check; it does on BrowserStack's Galaxy S26). TC_43-46 are HQ web checks (mobile workers page) - N/A for this mobile suite. The rest are not automatable, confirmed with the team 2026-10-23: TC_01-03 need an SMS OTP and there is no test number that receives one; TC_37-42 need fingerprint enrollment.</t>
+        </is>
+      </c>
+      <c r="J19" s="95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K19" s="95" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="95" t="n">
+        <v>46</v>
+      </c>
+      <c r="M19" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="95" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="100" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I20" s="101" t="inlineStr">
+        <is>
+          <t>85 of 209 test cases automated so far; 0 more assessed automatable; 118 not automatable; the rest N/A.</t>
+        </is>
+      </c>
+      <c r="K20" s="100" t="n">
+        <v>85</v>
+      </c>
+      <c r="L20" s="100" t="n">
+        <v>118</v>
+      </c>
+      <c r="M20" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="100" t="n">
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>